<commit_message>
Agrego una fila al dataset
</commit_message>
<xml_diff>
--- a/Dataset_preguntas_respuestas_gimnasio.xlsx
+++ b/Dataset_preguntas_respuestas_gimnasio.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="42">
   <si>
     <t>Preguntas</t>
   </si>
@@ -146,6 +146,9 @@
   </si>
   <si>
     <t>No se dictan clases de defensa personal.</t>
+  </si>
+  <si>
+    <t>¿Hay lockers para dejar las cosas?</t>
   </si>
 </sst>
 </file>
@@ -578,6 +581,14 @@
         <v>40</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Cargo el dataset para el gimnasio
</commit_message>
<xml_diff>
--- a/Dataset_preguntas_respuestas_gimnasio.xlsx
+++ b/Dataset_preguntas_respuestas_gimnasio.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="41">
   <si>
     <t>Preguntas</t>
   </si>
@@ -146,9 +146,6 @@
   </si>
   <si>
     <t>No se dictan clases de defensa personal.</t>
-  </si>
-  <si>
-    <t>¿Hay lockers para dejar las cosas?</t>
   </si>
 </sst>
 </file>
@@ -581,14 +578,6 @@
         <v>40</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>